<commit_message>
Sanitize performance score template sample IDs
</commit_message>
<xml_diff>
--- a/public/templates/performance-score-class-sheet-template.xlsx
+++ b/public/templates/performance-score-class-sheet-template.xlsx
@@ -834,8 +834,10 @@
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4">
-        <v>2024000272</v>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>S-001</t>
+        </is>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="11">
@@ -858,8 +860,10 @@
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4">
-        <v>2024000174</v>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>S-002</t>
+        </is>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="11">
@@ -882,8 +886,10 @@
       <c r="B9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="4">
-        <v>2024000311</v>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>S-003</t>
+        </is>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="11">
@@ -906,8 +912,10 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="4">
-        <v>2024000108</v>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>S-004</t>
+        </is>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="11">
@@ -930,8 +938,10 @@
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="4">
-        <v>2024000095</v>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>S-005</t>
+        </is>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="11">
@@ -954,8 +964,10 @@
       <c r="B12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="4">
-        <v>2024000049</v>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>S-006</t>
+        </is>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="11">
@@ -978,8 +990,10 @@
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="4">
-        <v>2024000038</v>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>S-007</t>
+        </is>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="11">
@@ -1002,8 +1016,10 @@
       <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="4">
-        <v>2024000294</v>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>S-008</t>
+        </is>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="11">
@@ -1026,8 +1042,10 @@
       <c r="B15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="4">
-        <v>2024000098</v>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>S-009</t>
+        </is>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="11">
@@ -1050,8 +1068,10 @@
       <c r="B16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="4">
-        <v>2024000290</v>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>S-010</t>
+        </is>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="11">
@@ -1074,8 +1094,10 @@
       <c r="B17" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="4">
-        <v>2024000026</v>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>S-011</t>
+        </is>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="11">
@@ -1098,8 +1120,10 @@
       <c r="B18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="4">
-        <v>2024000110</v>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>S-012</t>
+        </is>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="11">
@@ -1122,8 +1146,10 @@
       <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="4">
-        <v>2024000111</v>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>S-013</t>
+        </is>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="11">
@@ -1146,8 +1172,10 @@
       <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="4">
-        <v>2024000152</v>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>S-014</t>
+        </is>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="11">
@@ -1170,8 +1198,10 @@
       <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="4">
-        <v>2024000292</v>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>S-015</t>
+        </is>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="11">
@@ -1194,8 +1224,10 @@
       <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="4">
-        <v>2024000085</v>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>S-016</t>
+        </is>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="11">
@@ -1218,8 +1250,10 @@
       <c r="B23" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="4">
-        <v>2024000232</v>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>S-017</t>
+        </is>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="11">
@@ -1242,8 +1276,10 @@
       <c r="B24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="4">
-        <v>2024000244</v>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>S-018</t>
+        </is>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="11">
@@ -1266,8 +1302,10 @@
       <c r="B25" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="4">
-        <v>2024000323</v>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>S-019</t>
+        </is>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="11">
@@ -1290,8 +1328,10 @@
       <c r="B26" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="4">
-        <v>2024000288</v>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>S-020</t>
+        </is>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="11">
@@ -1314,8 +1354,10 @@
       <c r="B27" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="4">
-        <v>2024000122</v>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>S-021</t>
+        </is>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="11">
@@ -1338,8 +1380,10 @@
       <c r="B28" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="4">
-        <v>2024000010</v>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>S-022</t>
+        </is>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="11">
@@ -1362,8 +1406,10 @@
       <c r="B29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="4">
-        <v>2024000197</v>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="11">
@@ -1386,8 +1432,10 @@
       <c r="B30" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="4">
-        <v>2024000055</v>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="11">
@@ -1410,8 +1458,10 @@
       <c r="B31" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="4">
-        <v>2024000221</v>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>S-025</t>
+        </is>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="11">
@@ -1434,8 +1484,10 @@
       <c r="B32" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="4">
-        <v>2024000045</v>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>S-026</t>
+        </is>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="11">
@@ -1458,8 +1510,10 @@
       <c r="B33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="4">
-        <v>2024000297</v>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>S-027</t>
+        </is>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="11">
@@ -1482,8 +1536,10 @@
       <c r="B34" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="4">
-        <v>2024000116</v>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>S-028</t>
+        </is>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="11">
@@ -1506,8 +1562,10 @@
       <c r="B35" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="4">
-        <v>2024000173</v>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>S-029</t>
+        </is>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="11">
@@ -1530,8 +1588,10 @@
       <c r="B36" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="4">
-        <v>2024000188</v>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>S-030</t>
+        </is>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="11">
@@ -1554,8 +1614,10 @@
       <c r="B37" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="4">
-        <v>2025001409</v>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>S-031</t>
+        </is>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="11">
@@ -1578,8 +1640,10 @@
       <c r="B38" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="4">
-        <v>2024000309</v>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>S-032</t>
+        </is>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="11">

</xml_diff>